<commit_message>
calibrate voltage and current 2
</commit_message>
<xml_diff>
--- a/Calibration Data 2/Data/Voltage sensor/readings.xlsx
+++ b/Calibration Data 2/Data/Voltage sensor/readings.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kor\Documents\GitHub\Proa-II-Electrical-Setup\Calibration Data 2\Data\Voltage sensor\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Github\Proa-II-Electrical-Setup\Calibration Data 2\Data\Voltage sensor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{16D7BDBA-237B-4A18-83BE-650817777AA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDCC4E3D-BC38-4272-B85A-C4A85A3FB53F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{B6D28FCB-C6DA-474E-A13C-C90CDD553311}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{B6D28FCB-C6DA-474E-A13C-C90CDD553311}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Actual Voltage</t>
   </si>
@@ -53,9 +53,6 @@
     <t>Divided Voltage</t>
   </si>
   <si>
-    <t>Voltage Difference</t>
-  </si>
-  <si>
     <t>Average</t>
   </si>
   <si>
@@ -63,6 +60,18 @@
   </si>
   <si>
     <t>Ratio Adj</t>
+  </si>
+  <si>
+    <t>Actual Voltage Difference</t>
+  </si>
+  <si>
+    <t>Reading Voltage Difference</t>
+  </si>
+  <si>
+    <t>Reading Unit Difference</t>
+  </si>
+  <si>
+    <t>Offset Reading</t>
   </si>
 </sst>
 </file>
@@ -104,7 +113,13 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="3">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -180,7 +195,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Voltage Difference</c:v>
+                  <c:v>Actual Voltage Difference</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1285,16 +1300,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>45720</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>171450</xdr:rowOff>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>472440</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>11430</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>350520</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>171450</xdr:rowOff>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>167640</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>11430</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1323,9 +1338,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BFEBCCB0-9A45-4E14-BF66-68D32D6CCCDD}" name="Table1" displayName="Table1" ref="A1:F52" totalsRowShown="0">
-  <autoFilter ref="A1:F52" xr:uid="{BFEBCCB0-9A45-4E14-BF66-68D32D6CCCDD}"/>
-  <tableColumns count="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BFEBCCB0-9A45-4E14-BF66-68D32D6CCCDD}" name="Table1" displayName="Table1" ref="A1:H52" totalsRowShown="0">
+  <autoFilter ref="A1:H52" xr:uid="{BFEBCCB0-9A45-4E14-BF66-68D32D6CCCDD}"/>
+  <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{A3ADD35A-592E-4B27-B8B9-90526802A05C}" name="Actual Voltage"/>
     <tableColumn id="2" xr3:uid="{E82573D6-AD3C-49B1-9451-AA62B4394954}" name="Divided Voltage">
       <calculatedColumnFormula>A2/12</calculatedColumnFormula>
@@ -1334,11 +1349,17 @@
     <tableColumn id="4" xr3:uid="{7B4252B1-7BDF-4D58-8C5B-44B38564D29F}" name="ADS Voltage Reading">
       <calculatedColumnFormula>C2*0.0001875</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{F0F0EA9C-97E8-4599-8F32-A0AA4B58F728}" name="Scaled Voltage" dataDxfId="0">
-      <calculatedColumnFormula>D2*$I$3</calculatedColumnFormula>
+    <tableColumn id="5" xr3:uid="{F0F0EA9C-97E8-4599-8F32-A0AA4B58F728}" name="Scaled Voltage" dataDxfId="2">
+      <calculatedColumnFormula>D2*$L$3</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{756DED9B-96DF-4B2E-98FA-53567F8ACDC1}" name="Voltage Difference">
+    <tableColumn id="6" xr3:uid="{756DED9B-96DF-4B2E-98FA-53567F8ACDC1}" name="Actual Voltage Difference">
       <calculatedColumnFormula>A2-E2</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="7" xr3:uid="{A717BE8B-55E4-4512-8C2D-6F0B652DE131}" name="Reading Voltage Difference" dataDxfId="1">
+      <calculatedColumnFormula>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="8" xr3:uid="{699D0EAB-4BF1-4006-837D-EA8DB22A3E7C}" name="Reading Unit Difference" dataDxfId="0">
+      <calculatedColumnFormula>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1662,7 +1683,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6929F785-4062-4E0A-AC5E-7324F87C6CC8}">
-  <dimension ref="A1:I52"/>
+  <dimension ref="A1:L52"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.77734375" customWidth="1"/>
@@ -1670,10 +1691,13 @@
     <col min="3" max="3" width="18.33203125" customWidth="1"/>
     <col min="4" max="4" width="19.88671875" customWidth="1"/>
     <col min="5" max="5" width="17.6640625" customWidth="1"/>
-    <col min="6" max="6" width="18" customWidth="1"/>
+    <col min="6" max="6" width="24.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.77734375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1687,13 +1711,19 @@
         <v>2</v>
       </c>
       <c r="E1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+      <c r="G1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>55.2</v>
       </c>
@@ -1709,1232 +1739,1648 @@
         <v>4.5511875000000002</v>
       </c>
       <c r="E2">
-        <f t="shared" ref="E2:E33" si="0">D2*$I$3</f>
+        <f>D2*$L$3</f>
         <v>55.296928125000001</v>
       </c>
       <c r="F2">
         <f>A2-E2</f>
         <v>-9.6928124999998033E-2</v>
       </c>
-      <c r="H2" t="s">
-        <v>5</v>
-      </c>
-      <c r="I2">
+      <c r="G2">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>4.8812500000000369E-2</v>
+      </c>
+      <c r="H2">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>260.3333333333353</v>
+      </c>
+      <c r="K2" t="s">
+        <v>4</v>
+      </c>
+      <c r="L2">
         <f>AVERAGE(F:F)</f>
         <v>1.7806372548778268E-4</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>52.8</v>
       </c>
       <c r="B3">
-        <f t="shared" ref="B3:B52" si="1">A3/12</f>
+        <f t="shared" ref="B3:B52" si="0">A3/12</f>
         <v>4.3999999999999995</v>
       </c>
       <c r="C3">
         <v>23145</v>
       </c>
       <c r="D3">
-        <f t="shared" ref="D3:D52" si="2">C3*0.0001875</f>
+        <f t="shared" ref="D3:D52" si="1">C3*0.0001875</f>
         <v>4.3396875000000001</v>
       </c>
       <c r="E3">
-        <f t="shared" si="0"/>
+        <f>D3*$L$3</f>
         <v>52.727203125000003</v>
       </c>
       <c r="F3">
-        <f t="shared" ref="F3:F52" si="3">A3-E3</f>
+        <f t="shared" ref="F3:F52" si="2">A3-E3</f>
         <v>7.2796874999994543E-2</v>
       </c>
-      <c r="H3" t="s">
-        <v>7</v>
-      </c>
-      <c r="I3">
+      <c r="G3">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>6.0312499999999325E-2</v>
+      </c>
+      <c r="H3">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>321.66666666666305</v>
+      </c>
+      <c r="K3" t="s">
+        <v>6</v>
+      </c>
+      <c r="L3">
         <v>12.15</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>52.4</v>
       </c>
       <c r="B4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>4.3666666666666663</v>
       </c>
       <c r="C4">
         <v>22989</v>
       </c>
       <c r="D4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>4.3104374999999999</v>
       </c>
       <c r="E4">
-        <f t="shared" si="0"/>
+        <f>D4*$L$3</f>
         <v>52.371815625000004</v>
       </c>
       <c r="F4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>2.8184374999995043E-2</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G4">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>5.622916666666633E-2</v>
+      </c>
+      <c r="H4">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>299.8888888888871</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>53.6</v>
       </c>
       <c r="B5">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>4.4666666666666668</v>
       </c>
       <c r="C5">
         <v>23524</v>
       </c>
       <c r="D5">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>4.4107500000000002</v>
       </c>
       <c r="E5">
-        <f t="shared" si="0"/>
+        <f>D5*$L$3</f>
         <v>53.590612500000006</v>
       </c>
       <c r="F5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>9.3874999999954412E-3</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G5">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>5.5916666666666615E-2</v>
+      </c>
+      <c r="H5">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>298.22222222222194</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>53.9</v>
       </c>
       <c r="B6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>4.4916666666666663</v>
       </c>
       <c r="C6">
         <v>23690</v>
       </c>
       <c r="D6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>4.4418750000000005</v>
       </c>
       <c r="E6">
-        <f t="shared" si="0"/>
+        <f>D6*$L$3</f>
         <v>53.968781250000006</v>
       </c>
       <c r="F6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>-6.8781250000007788E-2</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G6">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>4.979166666666579E-2</v>
+      </c>
+      <c r="H6">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>265.55555555555088</v>
+      </c>
+      <c r="K6" t="s">
+        <v>10</v>
+      </c>
+      <c r="L6">
+        <f>AVERAGE(H:H)</f>
+        <v>247.55119825708005</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>54</v>
       </c>
       <c r="B7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>4.5</v>
       </c>
       <c r="C7">
         <v>23710</v>
       </c>
       <c r="D7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>4.4456249999999997</v>
       </c>
       <c r="E7">
-        <f t="shared" si="0"/>
+        <f>D7*$L$3</f>
         <v>54.014343749999995</v>
       </c>
       <c r="F7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>-1.434374999999477E-2</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G7">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>5.4375000000000284E-2</v>
+      </c>
+      <c r="H7">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>290.00000000000153</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>54</v>
       </c>
       <c r="B8">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>4.5</v>
       </c>
       <c r="C8">
         <v>23738</v>
       </c>
       <c r="D8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>4.4508749999999999</v>
       </c>
       <c r="E8">
-        <f t="shared" si="0"/>
+        <f>D8*$L$3</f>
         <v>54.078131249999998</v>
       </c>
       <c r="F8">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>-7.8131249999998431E-2</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G8">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>4.9125000000000085E-2</v>
+      </c>
+      <c r="H8">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>262.00000000000045</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>51.8</v>
       </c>
       <c r="B9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>4.3166666666666664</v>
       </c>
       <c r="C9">
         <v>22720</v>
       </c>
       <c r="D9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>4.26</v>
       </c>
       <c r="E9">
-        <f t="shared" si="0"/>
+        <f>D9*$L$3</f>
         <v>51.759</v>
       </c>
       <c r="F9">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>4.0999999999996817E-2</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G9">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>5.6666666666666643E-2</v>
+      </c>
+      <c r="H9">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>302.22222222222211</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>51.5</v>
       </c>
       <c r="B10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>4.291666666666667</v>
       </c>
       <c r="C10">
         <v>22609</v>
       </c>
       <c r="D10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>4.2391874999999999</v>
       </c>
       <c r="E10">
-        <f t="shared" si="0"/>
+        <f>D10*$L$3</f>
         <v>51.506128125000004</v>
       </c>
       <c r="F10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>-6.1281250000035925E-3</v>
       </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G10">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>5.2479166666667076E-2</v>
+      </c>
+      <c r="H10">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>279.88888888889107</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>53</v>
       </c>
       <c r="B11">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>4.416666666666667</v>
       </c>
       <c r="C11">
         <v>23276</v>
       </c>
       <c r="D11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>4.3642500000000002</v>
       </c>
       <c r="E11">
-        <f t="shared" si="0"/>
+        <f>D11*$L$3</f>
         <v>53.025637500000002</v>
       </c>
       <c r="F11">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>-2.5637500000001978E-2</v>
       </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G11">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>5.2416666666666778E-2</v>
+      </c>
+      <c r="H11">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>279.55555555555617</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>53.1</v>
       </c>
       <c r="B12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>4.4249999999999998</v>
       </c>
       <c r="C12">
         <v>23302</v>
       </c>
       <c r="D12">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>4.3691250000000004</v>
       </c>
       <c r="E12">
-        <f t="shared" si="0"/>
+        <f>D12*$L$3</f>
         <v>53.084868750000005</v>
       </c>
       <c r="F12">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>1.5131249999996044E-2</v>
       </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G12">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>5.5874999999999453E-2</v>
+      </c>
+      <c r="H12">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>297.9999999999971</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>53.1</v>
       </c>
       <c r="B13">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>4.4249999999999998</v>
       </c>
       <c r="C13">
         <v>23311</v>
       </c>
       <c r="D13">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>4.3708125000000004</v>
       </c>
       <c r="E13">
-        <f t="shared" si="0"/>
+        <f>D13*$L$3</f>
         <v>53.10537187500001</v>
       </c>
       <c r="F13">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>-5.3718750000086857E-3</v>
       </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G13">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>5.4187499999999389E-2</v>
+      </c>
+      <c r="H13">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>288.99999999999676</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>50.9</v>
       </c>
       <c r="B14">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>4.2416666666666663</v>
       </c>
       <c r="C14">
         <v>22354</v>
       </c>
       <c r="D14">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>4.1913749999999999</v>
       </c>
       <c r="E14">
-        <f t="shared" si="0"/>
+        <f>D14*$L$3</f>
         <v>50.925206250000002</v>
       </c>
       <c r="F14">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>-2.5206250000003649E-2</v>
       </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G14">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>5.0291666666666401E-2</v>
+      </c>
+      <c r="H14">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>268.22222222222081</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>52.1</v>
       </c>
       <c r="B15">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>4.3416666666666668</v>
       </c>
       <c r="C15">
         <v>22817</v>
       </c>
       <c r="D15">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>4.2781875000000005</v>
       </c>
       <c r="E15">
-        <f t="shared" si="0"/>
+        <f>D15*$L$3</f>
         <v>51.979978125000009</v>
       </c>
       <c r="F15">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0.12002187499999195</v>
       </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G15">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>6.3479166666666309E-2</v>
+      </c>
+      <c r="H15">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>338.55555555555367</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>52.3</v>
       </c>
       <c r="B16">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>4.3583333333333334</v>
       </c>
       <c r="C16">
         <v>22974</v>
       </c>
       <c r="D16">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>4.3076249999999998</v>
       </c>
       <c r="E16">
-        <f t="shared" si="0"/>
+        <f>D16*$L$3</f>
         <v>52.337643749999998</v>
       </c>
       <c r="F16">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>-3.7643750000000864E-2</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G16">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>5.0708333333333577E-2</v>
+      </c>
+      <c r="H16">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>270.44444444444576</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>52.4</v>
       </c>
       <c r="B17">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>4.3666666666666663</v>
       </c>
       <c r="C17">
         <v>22988</v>
       </c>
       <c r="D17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>4.3102499999999999</v>
       </c>
       <c r="E17">
-        <f t="shared" si="0"/>
+        <f>D17*$L$3</f>
         <v>52.3695375</v>
       </c>
       <c r="F17">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>3.0462499999998727E-2</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G17">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>5.6416666666666337E-2</v>
+      </c>
+      <c r="H17">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>300.88888888888715</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>50.9</v>
       </c>
       <c r="B18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>4.2416666666666663</v>
       </c>
       <c r="C18">
         <v>22329</v>
       </c>
       <c r="D18">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>4.1866874999999997</v>
       </c>
       <c r="E18">
-        <f t="shared" si="0"/>
+        <f>D18*$L$3</f>
         <v>50.868253124999995</v>
       </c>
       <c r="F18">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>3.1746875000003172E-2</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G18">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>5.4979166666666579E-2</v>
+      </c>
+      <c r="H18">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>293.22222222222177</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>50.4</v>
       </c>
       <c r="B19">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>4.2</v>
       </c>
       <c r="C19">
         <v>22107</v>
       </c>
       <c r="D19">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>4.1450624999999999</v>
       </c>
       <c r="E19">
-        <f t="shared" si="0"/>
+        <f>D19*$L$3</f>
         <v>50.362509375000002</v>
       </c>
       <c r="F19">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>3.7490624999996669E-2</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G19">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>5.4937500000000306E-2</v>
+      </c>
+      <c r="H19">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>293.00000000000165</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>50.2</v>
       </c>
       <c r="B20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>4.1833333333333336</v>
       </c>
       <c r="C20">
         <v>22031</v>
       </c>
       <c r="D20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>4.1308125000000002</v>
       </c>
       <c r="E20">
-        <f t="shared" si="0"/>
+        <f>D20*$L$3</f>
         <v>50.189371875000006</v>
       </c>
       <c r="F20">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>1.0628124999996658E-2</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G20">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>5.252083333333335E-2</v>
+      </c>
+      <c r="H20">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>280.1111111111112</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>51.4</v>
       </c>
       <c r="B21">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>4.2833333333333332</v>
       </c>
       <c r="C21">
         <v>22581</v>
       </c>
       <c r="D21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>4.2339374999999997</v>
       </c>
       <c r="E21">
-        <f t="shared" si="0"/>
+        <f>D21*$L$3</f>
         <v>51.442340625</v>
       </c>
       <c r="F21">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>-4.2340625000001353E-2</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G21">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>4.9395833333333528E-2</v>
+      </c>
+      <c r="H21">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>263.44444444444548</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>51.7</v>
       </c>
       <c r="B22">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>4.3083333333333336</v>
       </c>
       <c r="C22">
         <v>22695</v>
       </c>
       <c r="D22">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>4.2553125000000005</v>
       </c>
       <c r="E22">
-        <f t="shared" si="0"/>
+        <f>D22*$L$3</f>
         <v>51.702046875000008</v>
       </c>
       <c r="F22">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>-2.0468750000048885E-3</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G22">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>5.3020833333333073E-2</v>
+      </c>
+      <c r="H22">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>282.77777777777641</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>51.8</v>
       </c>
       <c r="B23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>4.3166666666666664</v>
       </c>
       <c r="C23">
         <v>22729</v>
       </c>
       <c r="D23">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>4.2616874999999999</v>
       </c>
       <c r="E23">
-        <f t="shared" si="0"/>
+        <f>D23*$L$3</f>
         <v>51.779503124999998</v>
       </c>
       <c r="F23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>2.0496874999999193E-2</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G23">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>5.4979166666666579E-2</v>
+      </c>
+      <c r="H23">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>293.22222222222177</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>49.8</v>
       </c>
       <c r="B24">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>4.1499999999999995</v>
       </c>
       <c r="C24">
         <v>21821</v>
       </c>
       <c r="D24">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>4.0914375000000005</v>
       </c>
       <c r="E24">
-        <f t="shared" si="0"/>
+        <f>D24*$L$3</f>
         <v>49.710965625000007</v>
       </c>
       <c r="F24">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>8.9034374999990007E-2</v>
       </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G24">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>5.8562499999998963E-2</v>
+      </c>
+      <c r="H24">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>312.3333333333278</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>49.6</v>
       </c>
       <c r="B25">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>4.1333333333333337</v>
       </c>
       <c r="C25">
         <v>21779</v>
       </c>
       <c r="D25">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>4.0835625000000002</v>
       </c>
       <c r="E25">
-        <f t="shared" si="0"/>
+        <f>D25*$L$3</f>
         <v>49.615284375000002</v>
       </c>
       <c r="F25">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>-1.5284375000000239E-2</v>
       </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G25">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>4.9770833333333542E-2</v>
+      </c>
+      <c r="H25">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>265.44444444444554</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>51.2</v>
       </c>
       <c r="B26">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>4.2666666666666666</v>
       </c>
       <c r="C26">
         <v>22446</v>
       </c>
       <c r="D26">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>4.2086250000000005</v>
       </c>
       <c r="E26">
-        <f t="shared" si="0"/>
+        <f>D26*$L$3</f>
         <v>51.134793750000007</v>
       </c>
       <c r="F26">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>6.5206249999995691E-2</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G26">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>5.8041666666666103E-2</v>
+      </c>
+      <c r="H26">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>309.55555555555253</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>51.2</v>
       </c>
       <c r="B27">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>4.2666666666666666</v>
       </c>
       <c r="C27">
         <v>22500</v>
       </c>
       <c r="D27">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>4.21875</v>
       </c>
       <c r="E27">
-        <f t="shared" si="0"/>
+        <f>D27*$L$3</f>
         <v>51.2578125</v>
       </c>
       <c r="F27">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>-5.7812499999997158E-2</v>
       </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G27">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>4.7916666666666607E-2</v>
+      </c>
+      <c r="H27">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>255.55555555555523</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>51.3</v>
       </c>
       <c r="B28">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>4.2749999999999995</v>
       </c>
       <c r="C28">
         <v>22519</v>
       </c>
       <c r="D28">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>4.2223125000000001</v>
       </c>
       <c r="E28">
-        <f t="shared" si="0"/>
+        <f>D28*$L$3</f>
         <v>51.301096875000006</v>
       </c>
       <c r="F28">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>-1.0968750000088789E-3</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G28">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>5.2687499999999332E-2</v>
+      </c>
+      <c r="H28">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>280.99999999999642</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>49.5</v>
       </c>
       <c r="B29">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>4.125</v>
       </c>
       <c r="C29">
         <v>21714</v>
       </c>
       <c r="D29">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>4.0713749999999997</v>
       </c>
       <c r="E29">
-        <f t="shared" si="0"/>
+        <f>D29*$L$3</f>
         <v>49.467206249999997</v>
       </c>
       <c r="F29">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>3.2793750000003286E-2</v>
       </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G29">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>5.3625000000000256E-2</v>
+      </c>
+      <c r="H29">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>286.00000000000136</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>50.7</v>
       </c>
       <c r="B30">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>4.2250000000000005</v>
       </c>
       <c r="C30">
         <v>22258</v>
       </c>
       <c r="D30">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>4.1733750000000001</v>
       </c>
       <c r="E30">
-        <f t="shared" si="0"/>
+        <f>D30*$L$3</f>
         <v>50.706506250000004</v>
       </c>
       <c r="F30">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>-6.5062500000010459E-3</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G30">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>5.1625000000000476E-2</v>
+      </c>
+      <c r="H30">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>275.33333333333587</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>50.8</v>
       </c>
       <c r="B31">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>4.2333333333333334</v>
       </c>
       <c r="C31">
         <v>22293</v>
       </c>
       <c r="D31">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>4.1799375000000003</v>
       </c>
       <c r="E31">
-        <f t="shared" si="0"/>
+        <f>D31*$L$3</f>
         <v>50.786240625000005</v>
       </c>
       <c r="F31">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>1.3759374999992247E-2</v>
       </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G31">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>5.3395833333333087E-2</v>
+      </c>
+      <c r="H31">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>284.77777777777646</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>50</v>
       </c>
       <c r="B32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>4.166666666666667</v>
       </c>
       <c r="C32">
         <v>21945</v>
       </c>
       <c r="D32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>4.1146875000000005</v>
       </c>
       <c r="E32">
-        <f t="shared" si="0"/>
+        <f>D32*$L$3</f>
         <v>49.993453125000009</v>
       </c>
       <c r="F32">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>6.5468749999908482E-3</v>
       </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G32">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>5.1979166666666465E-2</v>
+      </c>
+      <c r="H32">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>277.22222222222115</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>50.2</v>
       </c>
       <c r="B33">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>4.1833333333333336</v>
       </c>
       <c r="C33">
         <v>22034</v>
       </c>
       <c r="D33">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>4.1313750000000002</v>
       </c>
       <c r="E33">
-        <f t="shared" si="0"/>
+        <f>D33*$L$3</f>
         <v>50.196206250000003</v>
       </c>
       <c r="F33">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>3.7937499999998181E-3</v>
       </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G33">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>5.1958333333333329E-2</v>
+      </c>
+      <c r="H33">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>277.11111111111109</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>48.1</v>
       </c>
       <c r="B34">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>4.0083333333333337</v>
       </c>
       <c r="C34">
         <v>21102</v>
       </c>
       <c r="D34">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>3.9566250000000003</v>
       </c>
       <c r="E34">
-        <f t="shared" ref="E34:E65" si="4">D34*$I$3</f>
+        <f>D34*$L$3</f>
         <v>48.072993750000002</v>
       </c>
       <c r="F34">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>2.7006249999999454E-2</v>
       </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G34">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>5.1708333333333467E-2</v>
+      </c>
+      <c r="H34">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>275.77777777777851</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>49.4</v>
       </c>
       <c r="B35">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>4.1166666666666663</v>
       </c>
       <c r="C35">
         <v>21686</v>
       </c>
       <c r="D35">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>4.0661250000000004</v>
       </c>
       <c r="E35">
-        <f t="shared" si="4"/>
+        <f>D35*$L$3</f>
         <v>49.403418750000007</v>
       </c>
       <c r="F35">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>-3.4187500000086857E-3</v>
       </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G35">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>5.0541666666665819E-2</v>
+      </c>
+      <c r="H35">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>269.55555555555105</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>49.4</v>
       </c>
       <c r="B36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>4.1166666666666663</v>
       </c>
       <c r="C36">
         <v>21697</v>
       </c>
       <c r="D36">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>4.0681875000000005</v>
       </c>
       <c r="E36">
-        <f t="shared" si="4"/>
+        <f>D36*$L$3</f>
         <v>49.428478125000005</v>
       </c>
       <c r="F36">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>-2.8478125000006571E-2</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G36">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>4.8479166666665741E-2</v>
+      </c>
+      <c r="H36">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>258.5555555555506</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>47.6</v>
       </c>
       <c r="B37">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>3.9666666666666668</v>
       </c>
       <c r="C37">
         <v>20892</v>
       </c>
       <c r="D37">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>3.9172500000000001</v>
       </c>
       <c r="E37">
-        <f t="shared" si="4"/>
+        <f>D37*$L$3</f>
         <v>47.594587500000003</v>
       </c>
       <c r="F37">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>5.412499999998488E-3</v>
       </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G37">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>4.9416666666666664E-2</v>
+      </c>
+      <c r="H37">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>263.55555555555554</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>49.1</v>
       </c>
       <c r="B38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>4.0916666666666668</v>
       </c>
       <c r="C38">
         <v>21545</v>
       </c>
       <c r="D38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>4.0396875000000003</v>
       </c>
       <c r="E38">
-        <f t="shared" si="4"/>
+        <f>D38*$L$3</f>
         <v>49.082203125000007</v>
       </c>
       <c r="F38">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>1.7796874999994827E-2</v>
       </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G38">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>5.1979166666666465E-2</v>
+      </c>
+      <c r="H38">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>277.22222222222115</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>45.1</v>
       </c>
       <c r="B39">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>3.7583333333333333</v>
       </c>
       <c r="C39">
         <v>19864</v>
       </c>
       <c r="D39">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>3.7244999999999999</v>
       </c>
       <c r="E39">
-        <f t="shared" si="4"/>
+        <f>D39*$L$3</f>
         <v>45.252675000000004</v>
       </c>
       <c r="F39">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>-0.15267500000000211</v>
       </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G39">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>3.3833333333333382E-2</v>
+      </c>
+      <c r="H39">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>180.44444444444471</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>46.7</v>
       </c>
       <c r="B40">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>3.8916666666666671</v>
       </c>
       <c r="C40">
         <v>20495</v>
       </c>
       <c r="D40">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>3.8428125</v>
       </c>
       <c r="E40">
-        <f t="shared" si="4"/>
+        <f>D40*$L$3</f>
         <v>46.690171875000004</v>
       </c>
       <c r="F40">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>9.8281249999985221E-3</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G40">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>4.8854166666667087E-2</v>
+      </c>
+      <c r="H40">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>260.55555555555782</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>48.2</v>
       </c>
       <c r="B41">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>4.0166666666666666</v>
       </c>
       <c r="C41">
         <v>21172</v>
       </c>
       <c r="D41">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>3.9697499999999999</v>
       </c>
       <c r="E41">
-        <f t="shared" si="4"/>
+        <f>D41*$L$3</f>
         <v>48.232462499999997</v>
       </c>
       <c r="F41">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>-3.2462499999994066E-2</v>
       </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G41">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>4.6916666666666718E-2</v>
+      </c>
+      <c r="H41">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>250.22222222222248</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>21.3</v>
       </c>
       <c r="B42">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1.7750000000000001</v>
       </c>
       <c r="C42">
         <v>9291</v>
       </c>
       <c r="D42">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1.7420625000000001</v>
       </c>
       <c r="E42">
-        <f t="shared" si="4"/>
+        <f>D42*$L$3</f>
         <v>21.166059375000003</v>
       </c>
       <c r="F42">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0.13394062499999748</v>
       </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G42">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>3.2937500000000064E-2</v>
+      </c>
+      <c r="H42">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>175.666666666667</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>22.1</v>
       </c>
       <c r="B43">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1.8416666666666668</v>
       </c>
       <c r="C43">
         <v>9699</v>
       </c>
       <c r="D43">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1.8185625000000001</v>
       </c>
       <c r="E43">
-        <f t="shared" si="4"/>
+        <f>D43*$L$3</f>
         <v>22.095534375000003</v>
       </c>
       <c r="F43">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>4.4656249999981412E-3</v>
       </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G43">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>2.3104166666666703E-2</v>
+      </c>
+      <c r="H43">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>123.22222222222241</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>22.8</v>
       </c>
       <c r="B44">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1.9000000000000001</v>
       </c>
       <c r="C44">
         <v>10005</v>
       </c>
       <c r="D44">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1.8759375</v>
       </c>
       <c r="E44">
-        <f t="shared" si="4"/>
+        <f>D44*$L$3</f>
         <v>22.792640625000001</v>
       </c>
       <c r="F44">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>7.3593750000000568E-3</v>
       </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G44">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>2.4062500000000098E-2</v>
+      </c>
+      <c r="H44">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>128.33333333333385</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>23.5</v>
       </c>
       <c r="B45">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1.9583333333333333</v>
       </c>
       <c r="C45">
         <v>10301</v>
       </c>
       <c r="D45">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1.9314375000000001</v>
       </c>
       <c r="E45">
-        <f t="shared" si="4"/>
+        <f>D45*$L$3</f>
         <v>23.466965625000004</v>
       </c>
       <c r="F45">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>3.3034374999996174E-2</v>
       </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G45">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>2.6895833333333119E-2</v>
+      </c>
+      <c r="H45">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>143.44444444444329</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>23.3</v>
       </c>
       <c r="B46">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1.9416666666666667</v>
       </c>
       <c r="C46">
         <v>10240</v>
       </c>
       <c r="D46">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1.92</v>
       </c>
       <c r="E46">
-        <f t="shared" si="4"/>
+        <f>D46*$L$3</f>
         <v>23.327999999999999</v>
       </c>
       <c r="F46">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>-2.7999999999998693E-2</v>
       </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G46">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>2.1666666666666723E-2</v>
+      </c>
+      <c r="H46">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>115.55555555555586</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>24</v>
       </c>
       <c r="B47">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="C47">
         <v>10547</v>
       </c>
       <c r="D47">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1.9775625000000001</v>
       </c>
       <c r="E47">
-        <f t="shared" si="4"/>
+        <f>D47*$L$3</f>
         <v>24.027384375</v>
       </c>
       <c r="F47">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>-2.738437500000046E-2</v>
       </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G47">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>2.2437499999999888E-2</v>
+      </c>
+      <c r="H47">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>119.66666666666606</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>24.5</v>
       </c>
       <c r="B48">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>2.0416666666666665</v>
       </c>
       <c r="C48">
         <v>10773</v>
       </c>
       <c r="D48">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>2.0199375000000002</v>
       </c>
       <c r="E48">
-        <f t="shared" si="4"/>
+        <f>D48*$L$3</f>
         <v>24.542240625000002</v>
       </c>
       <c r="F48">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>-4.2240625000001586E-2</v>
       </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G48">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>2.1729166666666355E-2</v>
+      </c>
+      <c r="H48">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>115.88888888888722</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>24.3</v>
       </c>
       <c r="B49">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>2.0249999999999999</v>
       </c>
       <c r="C49">
         <v>10683</v>
       </c>
       <c r="D49">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>2.0030625</v>
       </c>
       <c r="E49">
-        <f t="shared" si="4"/>
+        <f>D49*$L$3</f>
         <v>24.337209375</v>
       </c>
       <c r="F49">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>-3.7209374999999767E-2</v>
       </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G49">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>2.1937499999999943E-2</v>
+      </c>
+      <c r="H49">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>116.99999999999969</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>24.8</v>
       </c>
       <c r="B50">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>2.0666666666666669</v>
       </c>
       <c r="C50">
         <v>10866</v>
       </c>
       <c r="D50">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>2.0373749999999999</v>
       </c>
       <c r="E50">
-        <f t="shared" si="4"/>
+        <f>D50*$L$3</f>
         <v>24.75410625</v>
       </c>
       <c r="F50">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>4.5893750000001177E-2</v>
       </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G50">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>2.9291666666666938E-2</v>
+      </c>
+      <c r="H50">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>156.22222222222368</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>24.5</v>
       </c>
       <c r="B51">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>2.0416666666666665</v>
       </c>
       <c r="C51">
         <v>10775</v>
       </c>
       <c r="D51">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>2.0203125000000002</v>
       </c>
       <c r="E51">
-        <f t="shared" si="4"/>
+        <f>D51*$L$3</f>
         <v>24.546796875000002</v>
       </c>
       <c r="F51">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>-4.6796875000001847E-2</v>
       </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G51">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>2.1354166666666341E-2</v>
+      </c>
+      <c r="H51">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>113.88888888888715</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>24.7</v>
       </c>
       <c r="B52">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>2.0583333333333331</v>
       </c>
       <c r="C52">
         <v>10852</v>
       </c>
       <c r="D52">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>2.0347499999999998</v>
       </c>
       <c r="E52">
-        <f t="shared" si="4"/>
+        <f>D52*$L$3</f>
         <v>24.722212499999998</v>
       </c>
       <c r="F52">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>-2.2212499999998414E-2</v>
+      </c>
+      <c r="G52">
+        <f>Table1[[#This Row],[Divided Voltage]]-Table1[[#This Row],[ADS Voltage Reading]]</f>
+        <v>2.358333333333329E-2</v>
+      </c>
+      <c r="H52">
+        <f>Table1[[#This Row],[Reading Voltage Difference]]/0.0001875</f>
+        <v>125.77777777777754</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>